<commit_message>
feat: harden email identity and finalize demo admin flow
</commit_message>
<xml_diff>
--- a/docs/datos-iniciales/PlayPredict_Base_Inicial_v1.0_2026-09-01.xlsx
+++ b/docs/datos-iniciales/PlayPredict_Base_Inicial_v1.0_2026-09-01.xlsx
@@ -420,7 +420,7 @@
         <x:v>Usuarios</x:v>
       </x:c>
       <x:c r="B6" s="24" t="str">
-        <x:v>Sólo ADMIN / admin123 y USUARIO / usuario. Contraseñas DEMO; no usar en producción.</x:v>
+        <x:v>Sólo admin@playpredict.local / admin123 y usuario@playpredict.local / usuario. Contraseñas DEMO; no usar en producción.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -428,7 +428,7 @@
         <x:v>Participación inicial</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
-        <x:v>USUARIO queda participante de COPA EL NENE.</x:v>
+        <x:v>usuario@playpredict.local queda participante de COPA EL NENE.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -641,7 +641,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="18" t="str">
-        <x:v>USUARIO</x:v>
+        <x:v>EMAIL</x:v>
       </x:c>
       <x:c r="B4" s="18" t="str">
         <x:v>ROL</x:v>
@@ -661,7 +661,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="24" t="str">
-        <x:v>ADMIN</x:v>
+        <x:v>admin@playpredict.local</x:v>
       </x:c>
       <x:c r="B5" s="24" t="str">
         <x:v>ADMIN</x:v>
@@ -681,7 +681,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="24" t="str">
-        <x:v>USUARIO</x:v>
+        <x:v>usuario@playpredict.local</x:v>
       </x:c>
       <x:c r="B6" s="24" t="str">
         <x:v>PLAYER</x:v>
@@ -736,7 +736,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="18" t="str">
-        <x:v>USUARIO</x:v>
+        <x:v>EMAIL</x:v>
       </x:c>
       <x:c r="B4" s="18" t="str">
         <x:v>COMPETENCIA_CODIGO</x:v>
@@ -750,7 +750,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="24" t="str">
-        <x:v>USUARIO</x:v>
+        <x:v>usuario@playpredict.local</x:v>
       </x:c>
       <x:c r="B5" s="24" t="str">
         <x:v>COPA_EL_NENE</x:v>

</xml_diff>